<commit_message>
fix: add status=已启用 for negative keywords
</commit_message>
<xml_diff>
--- a/ads_bulk_update.xlsx
+++ b/ads_bulk_update.xlsx
@@ -804,6 +804,11 @@
           <t>W12自动广告</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>已启用</t>
+        </is>
+      </c>
       <c r="T9" t="inlineStr">
         <is>
           <t>microwave</t>
@@ -841,6 +846,11 @@
           <t>W12自动广告</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>已启用</t>
+        </is>
+      </c>
       <c r="T10" t="inlineStr">
         <is>
           <t>kitchen storage</t>
@@ -878,6 +888,11 @@
           <t>W12自动广告</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>已启用</t>
+        </is>
+      </c>
       <c r="T11" t="inlineStr">
         <is>
           <t>b07vwr8vj1</t>
@@ -915,6 +930,11 @@
           <t>W12自动广告</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>已启用</t>
+        </is>
+      </c>
       <c r="T12" t="inlineStr">
         <is>
           <t>b0f89nh63r</t>
@@ -952,6 +972,11 @@
           <t>W14新品自动广告</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>已启用</t>
+        </is>
+      </c>
       <c r="T13" t="inlineStr">
         <is>
           <t>meat grinder</t>
@@ -989,6 +1014,11 @@
           <t>W14新品自动广告</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>已启用</t>
+        </is>
+      </c>
       <c r="T14" t="inlineStr">
         <is>
           <t>juicer</t>
@@ -1026,6 +1056,11 @@
           <t>压肉板自动广告</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>已启用</t>
+        </is>
+      </c>
       <c r="T15" t="inlineStr">
         <is>
           <t>cast iron burger press</t>
@@ -1061,6 +1096,11 @@
       <c r="J16" t="inlineStr">
         <is>
           <t>压肉板自动广告</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>已启用</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">

</xml_diff>